<commit_message>
add verwerking data (incl nog foute berekeningen :()
</commit_message>
<xml_diff>
--- a/Data/Kalibratie_magnetisch_veld.xlsx
+++ b/Data/Kalibratie_magnetisch_veld.xlsx
@@ -8,21 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tristancools/Documents/Arduino/Project-experimenteren2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{550AD411-C9A4-C34F-9FEC-8510C193991F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA68CDCD-951D-C84E-BFA6-27C1B1B32CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="500" windowWidth="25380" windowHeight="15640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kalibratie" sheetId="1" r:id="rId1"/>
     <sheet name="Metingen" sheetId="3" r:id="rId2"/>
     <sheet name="Verwerking" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>d(cm)</t>
   </si>
@@ -68,12 +81,122 @@
   <si>
     <t>V_AMPLIT (V)</t>
   </si>
+  <si>
+    <t>Meting:</t>
+  </si>
+  <si>
+    <t>Set 1</t>
+  </si>
+  <si>
+    <t>Set  2</t>
+  </si>
+  <si>
+    <t>Set 3</t>
+  </si>
+  <si>
+    <t>Set 4</t>
+  </si>
+  <si>
+    <t>Set 5</t>
+  </si>
+  <si>
+    <t>(Delta V_AC)_rms</t>
+  </si>
+  <si>
+    <t>V_CD = V_MAX (V)</t>
+  </si>
+  <si>
+    <t>Delta V_AC (V)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">V_piek = (Delta V_AC)_rms </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="5"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>want lockin meet rms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (V)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Draaihoek (radialen)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> (=Delta(V_AC)/(2V_DC)) </t>
+    </r>
+  </si>
+  <si>
+    <t>lengte kwarts (mm)</t>
+  </si>
+  <si>
+    <t>AF(lengte) (mm)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">R </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>(=V_max/I) (Ohm) (stroom van magnetisch veld, niet laser...)</t>
+    </r>
+  </si>
+  <si>
+    <t>B_veld door staaf (T*mm)</t>
+  </si>
+  <si>
+    <t>B_veld (mT) zie interpolatie python</t>
+  </si>
+  <si>
+    <t>B_veld door staaf (T*m)</t>
+  </si>
+  <si>
+    <t>Verdet-cste V (rad/Tm)</t>
+  </si>
+  <si>
+    <t>Verdet (graden/(T*m))</t>
+  </si>
+  <si>
+    <r>
+      <t>Draaihoek (graden)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> (=Delta(V_AC)/(2V_DC)) </t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,6 +210,24 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u val="double"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="5"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -96,7 +237,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -119,15 +260,65 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalDown="1">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal style="thin">
+        <color auto="1"/>
+      </diagonal>
+    </border>
+    <border diagonalDown="1">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="thin">
+        <color auto="1"/>
+      </diagonal>
+    </border>
+    <border diagonalDown="1">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="thin">
+        <color auto="1"/>
+      </diagonal>
+    </border>
+    <border diagonalDown="1">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal style="thin">
+        <color auto="1"/>
+      </diagonal>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,6 +623,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -2266,7 +2465,7 @@
         <v>1.2809999999999999</v>
       </c>
       <c r="F24">
-        <v>1.7</v>
+        <v>1.27</v>
       </c>
       <c r="G24">
         <v>2.5139999999999998</v>
@@ -2325,9 +2524,1538 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <f>Metingen!E2-Metingen!F2</f>
+        <v>1.6999999999999904E-2</v>
+      </c>
+      <c r="D2">
+        <f>C2/2</f>
+        <v>8.499999999999952E-3</v>
+      </c>
+      <c r="E2" s="3">
+        <f>2^(-1/2)*D2</f>
+        <v>6.0104076400856197E-3</v>
+      </c>
+      <c r="F2" s="6">
+        <f>Metingen!E2/(Metingen!C2*10^(-3))</f>
+        <v>19.719188767550705</v>
+      </c>
+      <c r="G2">
+        <f>Metingen!E2</f>
+        <v>1.264</v>
+      </c>
+      <c r="H2">
+        <f>D2/(2*G2)</f>
+        <v>3.3623417721518798E-3</v>
+      </c>
+      <c r="I2">
+        <f>H2/PI()*180</f>
+        <v>0.19264799282484057</v>
+      </c>
+      <c r="J2">
+        <v>200</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <f>(M2/J2)*10^(3)</f>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M2">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N2">
+        <f>M2*(10^(-3))</f>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O2">
+        <f>H2/N2</f>
+        <v>20.783608779233223</v>
+      </c>
+      <c r="P2">
+        <f>I2/N2</f>
+        <v>1190.8130661011087</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <f>Metingen!E3-Metingen!F3</f>
+        <v>2.0000000000000018E-2</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D26" si="0">C3/2</f>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="E3" s="3">
+        <f t="shared" ref="E3:E26" si="1">2^(-1/2)*D3</f>
+        <v>7.0710678118654805E-3</v>
+      </c>
+      <c r="F3" s="6">
+        <f>Metingen!E3/(Metingen!C3*10^(-3))</f>
+        <v>19.567233384853168</v>
+      </c>
+      <c r="G3">
+        <f>Metingen!E3</f>
+        <v>1.266</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H26" si="2">D3/(2*G3)</f>
+        <v>3.9494470774091659E-3</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I26" si="3">H3/PI()*180</f>
+        <v>0.22628664894582295</v>
+      </c>
+      <c r="J3">
+        <v>200</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <f t="shared" ref="L3:L26" si="4">(M3/J3)*10^(3)</f>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M3">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N26" si="5">M3*(10^(-3))</f>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O3">
+        <f t="shared" ref="O3:O26" si="6">H3/N3</f>
+        <v>24.412676793003406</v>
+      </c>
+      <c r="P3">
+        <f t="shared" ref="P3:P26" si="7">I3/N3</f>
+        <v>1398.7433468560648</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <f>Metingen!E4-Metingen!F4</f>
+        <v>2.0000000000000018E-2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="E4" s="3">
+        <f t="shared" si="1"/>
+        <v>7.0710678118654805E-3</v>
+      </c>
+      <c r="F4" s="6">
+        <f>Metingen!E4/(Metingen!C4*10^(-3))</f>
+        <v>19.656786271450862</v>
+      </c>
+      <c r="G4">
+        <f>Metingen!E4</f>
+        <v>1.26</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="2"/>
+        <v>3.9682539682539715E-3</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="3"/>
+        <v>0.22736420441699354</v>
+      </c>
+      <c r="J4">
+        <v>200</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M4">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O4">
+        <f t="shared" si="6"/>
+        <v>24.528927634874851</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="7"/>
+        <v>1405.4040294601414</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <f>Metingen!E5-Metingen!F5</f>
+        <v>2.4999999999999911E-2</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>1.2499999999999956E-2</v>
+      </c>
+      <c r="E5" s="3">
+        <f t="shared" si="1"/>
+        <v>8.838834764831811E-3</v>
+      </c>
+      <c r="F5" s="6">
+        <f>Metingen!E5/(Metingen!C5*10^(-3))</f>
+        <v>19.984375</v>
+      </c>
+      <c r="G5">
+        <f>Metingen!E5</f>
+        <v>1.2789999999999999</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="2"/>
+        <v>4.886630179827974E-3</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="3"/>
+        <v>0.27998328534539746</v>
+      </c>
+      <c r="J5">
+        <v>200</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M5">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="6"/>
+        <v>30.205677110967727</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="7"/>
+        <v>1730.6578157933648</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <f>Metingen!E6-Metingen!F6</f>
+        <v>2.4999999999999911E-2</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>1.2499999999999956E-2</v>
+      </c>
+      <c r="E6" s="3">
+        <f t="shared" si="1"/>
+        <v>8.838834764831811E-3</v>
+      </c>
+      <c r="F6" s="6">
+        <f>Metingen!E6/(Metingen!C6*10^(-3))</f>
+        <v>25.696969696969695</v>
+      </c>
+      <c r="G6">
+        <f>Metingen!E6</f>
+        <v>1.272</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="2"/>
+        <v>4.9135220125785988E-3</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>0.28152407386537992</v>
+      </c>
+      <c r="J6">
+        <v>200</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M6">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="6"/>
+        <v>30.371903321484055</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="7"/>
+        <v>1740.1818761004031</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <f>Metingen!E7-Metingen!F7</f>
+        <v>1.8000000000000016E-2</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>9.000000000000008E-3</v>
+      </c>
+      <c r="E7" s="3">
+        <f t="shared" si="1"/>
+        <v>6.3639610306789329E-3</v>
+      </c>
+      <c r="F7" s="6">
+        <f>Metingen!E7/(Metingen!C7*10^(-3))</f>
+        <v>21.805555555555554</v>
+      </c>
+      <c r="G7">
+        <f>Metingen!E7</f>
+        <v>1.256</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>3.5828025477707037E-3</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>0.20527946481597983</v>
+      </c>
+      <c r="J7">
+        <v>200</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M7">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="6"/>
+        <v>22.146340714926815</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="7"/>
+        <v>1268.8918546240448</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <f>Metingen!E8-Metingen!F8</f>
+        <v>1.8000000000000016E-2</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>9.000000000000008E-3</v>
+      </c>
+      <c r="E8" s="3">
+        <f t="shared" si="1"/>
+        <v>6.3639610306789329E-3</v>
+      </c>
+      <c r="F8" s="6">
+        <f>Metingen!E8/(Metingen!C8*10^(-3))</f>
+        <v>21.986062717770036</v>
+      </c>
+      <c r="G8">
+        <f>Metingen!E8</f>
+        <v>1.262</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="2"/>
+        <v>3.5657686212361363E-3</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>0.2043034927170132</v>
+      </c>
+      <c r="J8">
+        <v>200</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M8">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="6"/>
+        <v>22.041049079198164</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="7"/>
+        <v>1262.8590882787639</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <f>Metingen!E9-Metingen!F9</f>
+        <v>2.0000000000000018E-2</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="E9" s="3">
+        <f t="shared" si="1"/>
+        <v>7.0710678118654805E-3</v>
+      </c>
+      <c r="F9" s="6">
+        <f>Metingen!E9/(Metingen!C9*10^(-3))</f>
+        <v>21.6580310880829</v>
+      </c>
+      <c r="G9">
+        <f>Metingen!E9</f>
+        <v>1.254</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="2"/>
+        <v>3.9872408293460957E-3</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>0.22845207142377341</v>
+      </c>
+      <c r="J9">
+        <v>200</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M9">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="6"/>
+        <v>24.646290924993867</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="7"/>
+        <v>1412.1284506537304</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10">
+        <f>Metingen!E10-Metingen!F10</f>
+        <v>1.9999999999999796E-2</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>9.9999999999998979E-3</v>
+      </c>
+      <c r="E10" s="3">
+        <f t="shared" si="1"/>
+        <v>7.0710678118654025E-3</v>
+      </c>
+      <c r="F10" s="6">
+        <f>Metingen!E10/(Metingen!C10*10^(-3))</f>
+        <v>21.678200692041521</v>
+      </c>
+      <c r="G10">
+        <f>Metingen!E10</f>
+        <v>1.2529999999999999</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>3.9904229848363526E-3</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>0.22863439550311951</v>
+      </c>
+      <c r="J10">
+        <v>200</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M10">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="6"/>
+        <v>24.665960750153211</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="7"/>
+        <v>1413.2554486191211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <f>Metingen!E11-Metingen!F11</f>
+        <v>1.6999999999999904E-2</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>8.499999999999952E-3</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" si="1"/>
+        <v>6.0104076400856197E-3</v>
+      </c>
+      <c r="F11" s="6">
+        <f>Metingen!E11/(Metingen!C11*10^(-3))</f>
+        <v>30.071599045346062</v>
+      </c>
+      <c r="G11">
+        <f>Metingen!E11</f>
+        <v>1.26</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="2"/>
+        <v>3.3730158730158541E-3</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>0.19325957375444328</v>
+      </c>
+      <c r="J11">
+        <v>200</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M11">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="6"/>
+        <v>20.849588489643487</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="7"/>
+        <v>1194.5934250411124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <f>Metingen!E12-Metingen!F12</f>
+        <v>2.0999999999999908E-2</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>1.0499999999999954E-2</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" si="1"/>
+        <v>7.4246212024587158E-3</v>
+      </c>
+      <c r="F12" s="6">
+        <f>Metingen!E12/(Metingen!C12*10^(-3))</f>
+        <v>16.442432082794308</v>
+      </c>
+      <c r="G12">
+        <f>Metingen!E12</f>
+        <v>1.2709999999999999</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="2"/>
+        <v>4.1306058221872366E-3</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>0.23666628044349403</v>
+      </c>
+      <c r="J12">
+        <v>200</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M12">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="6"/>
+        <v>25.532471487757089</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="7"/>
+        <v>1462.9028567865912</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <f>Metingen!E13-Metingen!F13</f>
+        <v>2.200000000000002E-2</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>1.100000000000001E-2</v>
+      </c>
+      <c r="E13" s="3">
+        <f t="shared" si="1"/>
+        <v>7.778174593052029E-3</v>
+      </c>
+      <c r="F13" s="6">
+        <f>Metingen!E13/(Metingen!C13*10^(-3))</f>
+        <v>16.614785992217897</v>
+      </c>
+      <c r="G13">
+        <f>Metingen!E13</f>
+        <v>1.2809999999999999</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>4.2935206869633138E-3</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>0.24600061461510778</v>
+      </c>
+      <c r="J13">
+        <v>200</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M13">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="6"/>
+        <v>26.539495473799018</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="7"/>
+        <v>1520.601081055235</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <f>Metingen!E14-Metingen!F14</f>
+        <v>2.2999999999999909E-2</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="0"/>
+        <v>1.1499999999999955E-2</v>
+      </c>
+      <c r="E14" s="3">
+        <f t="shared" si="1"/>
+        <v>8.1317279836452643E-3</v>
+      </c>
+      <c r="F14" s="6">
+        <f>Metingen!E14/(Metingen!C14*10^(-3))</f>
+        <v>16.64072632944228</v>
+      </c>
+      <c r="G14">
+        <f>Metingen!E14</f>
+        <v>1.2829999999999999</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>4.4816835541698968E-3</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>0.25678155276712555</v>
+      </c>
+      <c r="J14">
+        <v>200</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M14">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="6"/>
+        <v>27.70258467882579</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="7"/>
+        <v>1587.241183700495</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15">
+        <f>Metingen!E15-Metingen!F15</f>
+        <v>2.8999999999999915E-2</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="0"/>
+        <v>1.4499999999999957E-2</v>
+      </c>
+      <c r="E15" s="3">
+        <f t="shared" si="1"/>
+        <v>1.0253048327204908E-2</v>
+      </c>
+      <c r="F15" s="6">
+        <f>Metingen!E15/(Metingen!C15*10^(-3))</f>
+        <v>16.579634464751958</v>
+      </c>
+      <c r="G15">
+        <f>Metingen!E15</f>
+        <v>1.27</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>5.7086614173228181E-3</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>0.32708220588176823</v>
+      </c>
+      <c r="J15">
+        <v>200</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M15">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O15">
+        <f t="shared" si="6"/>
+        <v>35.286890384973375</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="7"/>
+        <v>2021.789891199739</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <f>Metingen!E16-Metingen!F16</f>
+        <v>1.9000000000000128E-2</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>9.5000000000000639E-3</v>
+      </c>
+      <c r="E16" s="3">
+        <f t="shared" si="1"/>
+        <v>6.7175144212722462E-3</v>
+      </c>
+      <c r="F16" s="6">
+        <f>Metingen!E16/(Metingen!C16*10^(-3))</f>
+        <v>37.068965517241381</v>
+      </c>
+      <c r="G16">
+        <f>Metingen!E16</f>
+        <v>1.29</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="2"/>
+        <v>3.6821705426356836E-3</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>0.21097283154042085</v>
+      </c>
+      <c r="J16">
+        <v>200</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M16">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="6"/>
+        <v>22.760563084453775</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="7"/>
+        <v>1304.0842040804646</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <f>Metingen!E17-Metingen!F17</f>
+        <v>1.6000000000000014E-2</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>8.0000000000000071E-3</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" si="1"/>
+        <v>5.6568542494923844E-3</v>
+      </c>
+      <c r="F17" s="6">
+        <f>Metingen!E17/(Metingen!C17*10^(-3))</f>
+        <v>25.279999999999998</v>
+      </c>
+      <c r="G17">
+        <f>Metingen!E17</f>
+        <v>1.264</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="2"/>
+        <v>3.1645569620253194E-3</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>0.18131575795279234</v>
+      </c>
+      <c r="J17">
+        <v>200</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M17">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="6"/>
+        <v>19.561043556925515</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="7"/>
+        <v>1120.765238683404</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18">
+        <f>Metingen!E18-Metingen!F18</f>
+        <v>1.8000000000000016E-2</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>9.000000000000008E-3</v>
+      </c>
+      <c r="E18" s="3">
+        <f t="shared" si="1"/>
+        <v>6.3639610306789329E-3</v>
+      </c>
+      <c r="F18" s="6">
+        <f>Metingen!E18/(Metingen!C18*10^(-3))</f>
+        <v>25.568862275449096</v>
+      </c>
+      <c r="G18">
+        <f>Metingen!E18</f>
+        <v>1.2809999999999999</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="2"/>
+        <v>3.5128805620608934E-3</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>0.20127323013963366</v>
+      </c>
+      <c r="J18">
+        <v>200</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M18">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="6"/>
+        <v>21.714132660381019</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="7"/>
+        <v>1244.1281572270107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <f>Metingen!E19-Metingen!F19</f>
+        <v>1.9000000000000128E-2</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>9.5000000000000639E-3</v>
+      </c>
+      <c r="E19" s="3">
+        <f t="shared" si="1"/>
+        <v>6.7175144212722462E-3</v>
+      </c>
+      <c r="F19" s="6">
+        <f>Metingen!E19/(Metingen!C19*10^(-3))</f>
+        <v>25.64</v>
+      </c>
+      <c r="G19">
+        <f>Metingen!E19</f>
+        <v>1.282</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>3.705148205928262E-3</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>0.21228935467015825</v>
+      </c>
+      <c r="J19">
+        <v>200</v>
+      </c>
+      <c r="K19">
+        <v>1</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M19">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="6"/>
+        <v>22.902594679364562</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="7"/>
+        <v>1312.2220150263643</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>4</v>
+      </c>
+      <c r="C20">
+        <f>Metingen!E20-Metingen!F20</f>
+        <v>1.9000000000000128E-2</v>
+      </c>
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>9.5000000000000639E-3</v>
+      </c>
+      <c r="E20" s="3">
+        <f t="shared" si="1"/>
+        <v>6.7175144212722462E-3</v>
+      </c>
+      <c r="F20" s="6">
+        <f>Metingen!E20/(Metingen!C20*10^(-3))</f>
+        <v>25.72</v>
+      </c>
+      <c r="G20">
+        <f>Metingen!E20</f>
+        <v>1.286</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="2"/>
+        <v>3.6936236391913158E-3</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>0.21162904563541438</v>
+      </c>
+      <c r="J20">
+        <v>200</v>
+      </c>
+      <c r="K20">
+        <v>1</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M20">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="6"/>
+        <v>22.831357992959074</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="7"/>
+        <v>1308.140453548833</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <f>Metingen!E21-Metingen!F21</f>
+        <v>1.3000000000000123E-2</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>6.5000000000000613E-3</v>
+      </c>
+      <c r="E21" s="3">
+        <f t="shared" si="1"/>
+        <v>4.5961940777126016E-3</v>
+      </c>
+      <c r="F21" s="6">
+        <f>Metingen!E21/(Metingen!C21*10^(-3))</f>
+        <v>49.042145593869726</v>
+      </c>
+      <c r="G21">
+        <f>Metingen!E21</f>
+        <v>1.28</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>2.5390625000000239E-3</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
+        <v>0.14547756516993696</v>
+      </c>
+      <c r="J21">
+        <v>200</v>
+      </c>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M21">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="6"/>
+        <v>15.694681041377089</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="7"/>
+        <v>899.23898447489501</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <f>Metingen!E22-Metingen!F22</f>
+        <v>1.1999999999999789E-2</v>
+      </c>
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>5.9999999999998943E-3</v>
+      </c>
+      <c r="E22" s="3">
+        <f t="shared" si="1"/>
+        <v>4.2426406871192103E-3</v>
+      </c>
+      <c r="F22" s="6">
+        <f>Metingen!E22/(Metingen!C22*10^(-3))</f>
+        <v>41.213114754098356</v>
+      </c>
+      <c r="G22">
+        <f>Metingen!E22</f>
+        <v>1.2569999999999999</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="2"/>
+        <v>2.3866348448686931E-3</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>0.1367441038498361</v>
+      </c>
+      <c r="J22">
+        <v>200</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M22">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="6"/>
+        <v>14.752481536965032</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="7"/>
+        <v>845.25492941276639</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23">
+        <f>Metingen!E23-Metingen!F23</f>
+        <v>1.3000000000000123E-2</v>
+      </c>
+      <c r="D23">
+        <f t="shared" si="0"/>
+        <v>6.5000000000000613E-3</v>
+      </c>
+      <c r="E23" s="3">
+        <f t="shared" si="1"/>
+        <v>4.5961940777126016E-3</v>
+      </c>
+      <c r="F23" s="6">
+        <f>Metingen!E23/(Metingen!C23*10^(-3))</f>
+        <v>41.78217821782178</v>
+      </c>
+      <c r="G23">
+        <f>Metingen!E23</f>
+        <v>1.266</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="2"/>
+        <v>2.56714060031598E-3</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>0.14708632181478618</v>
+      </c>
+      <c r="J23">
+        <v>200</v>
+      </c>
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M23">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="6"/>
+        <v>15.868239915452349</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="7"/>
+        <v>909.18317545644993</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24">
+        <f>Metingen!E24-Metingen!F24</f>
+        <v>1.0999999999999899E-2</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="0"/>
+        <v>5.4999999999999494E-3</v>
+      </c>
+      <c r="E24" s="3">
+        <f t="shared" si="1"/>
+        <v>3.8890872965259751E-3</v>
+      </c>
+      <c r="F24" s="6">
+        <f>Metingen!E24/(Metingen!C24*10^(-3))</f>
+        <v>42.699999999999996</v>
+      </c>
+      <c r="G24">
+        <f>Metingen!E24</f>
+        <v>1.2809999999999999</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="2"/>
+        <v>2.1467603434816352E-3</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>0.12300030730755264</v>
+      </c>
+      <c r="J24">
+        <v>200</v>
+      </c>
+      <c r="K24">
+        <v>1</v>
+      </c>
+      <c r="L24">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M24">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="6"/>
+        <v>13.269747736899376</v>
+      </c>
+      <c r="P24">
+        <f t="shared" si="7"/>
+        <v>760.30054052760977</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="C25">
+        <f>Metingen!E25-Metingen!F25</f>
+        <v>1.2000000000000011E-2</v>
+      </c>
+      <c r="D25">
+        <f t="shared" si="0"/>
+        <v>6.0000000000000053E-3</v>
+      </c>
+      <c r="E25" s="3">
+        <f t="shared" si="1"/>
+        <v>4.2426406871192883E-3</v>
+      </c>
+      <c r="F25" s="6">
+        <f>Metingen!E25/(Metingen!C25*10^(-3))</f>
+        <v>42.400000000000006</v>
+      </c>
+      <c r="G25">
+        <f>Metingen!E25</f>
+        <v>1.272</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="2"/>
+        <v>2.3584905660377379E-3</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
+        <v>0.13513155545538297</v>
+      </c>
+      <c r="J25">
+        <v>200</v>
+      </c>
+      <c r="K25">
+        <v>1</v>
+      </c>
+      <c r="L25">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M25">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O25">
+        <f t="shared" si="6"/>
+        <v>14.578513594312412</v>
+      </c>
+      <c r="P25">
+        <f t="shared" si="7"/>
+        <v>835.28730052819731</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>5</v>
+      </c>
+      <c r="C26">
+        <f>Metingen!E26-Metingen!F26</f>
+        <v>1.0999999999999899E-2</v>
+      </c>
+      <c r="D26">
+        <f t="shared" si="0"/>
+        <v>5.4999999999999494E-3</v>
+      </c>
+      <c r="E26" s="4">
+        <f t="shared" si="1"/>
+        <v>3.8890872965259751E-3</v>
+      </c>
+      <c r="F26" s="6">
+        <f>Metingen!E26/(Metingen!C26*10^(-3))</f>
+        <v>62.749999999999993</v>
+      </c>
+      <c r="G26">
+        <f>Metingen!E26</f>
+        <v>1.2549999999999999</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="2"/>
+        <v>2.1912350597609364E-3</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="3"/>
+        <v>0.12554852084539839</v>
+      </c>
+      <c r="J26">
+        <v>200</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26">
+        <f t="shared" si="4"/>
+        <v>0.808892673035565</v>
+      </c>
+      <c r="M26">
+        <v>0.161778534607113</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="5"/>
+        <v>1.6177853460711301E-4</v>
+      </c>
+      <c r="O26">
+        <f t="shared" si="6"/>
+        <v>13.544658845392911</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="7"/>
+        <v>776.05178678555251</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>